<commit_message>
Harmonized USA and United States
</commit_message>
<xml_diff>
--- a/data/bugbook_data.xlsx
+++ b/data/bugbook_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thoma\Documents\Github\bugbook\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E243BC6-8680-4AD2-A686-F65B369C2BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44A1675D-C8A3-4C9C-A43F-8DCA0B0408B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="511">
   <si>
     <t>Chapter</t>
   </si>
@@ -823,9 +823,6 @@
   </si>
   <si>
     <t>Waterford</t>
-  </si>
-  <si>
-    <t>USA</t>
   </si>
   <si>
     <t>Ireland</t>
@@ -2126,13 +2123,13 @@
         <v>1</v>
       </c>
       <c r="D1" s="10" t="s">
+        <v>309</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>310</v>
       </c>
-      <c r="E1" s="10" t="s">
-        <v>311</v>
-      </c>
       <c r="F1" s="10" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G1" s="9" t="s">
         <v>15</v>
@@ -2152,10 +2149,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>304</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>305</v>
       </c>
       <c r="D2" s="5">
         <v>45627</v>
@@ -2167,13 +2164,13 @@
         <v>45838</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" t="s">
         <v>307</v>
-      </c>
-      <c r="I2" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
@@ -2184,7 +2181,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D3" s="5">
         <v>45632</v>
@@ -2228,16 +2225,16 @@
         <v>45832</v>
       </c>
       <c r="G4" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>300</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -2260,16 +2257,16 @@
         <v>45968</v>
       </c>
       <c r="G5" s="3" t="s">
+        <v>500</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>502</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>503</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>504</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -2327,13 +2324,13 @@
         <v>165</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>166</v>
       </c>
       <c r="J7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
@@ -2356,16 +2353,16 @@
         <v>45833</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>19</v>
       </c>
       <c r="I8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
@@ -2388,16 +2385,16 @@
         <v>45842</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>20</v>
       </c>
       <c r="I9" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
@@ -2423,7 +2420,7 @@
         <v>62</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>63</v>
@@ -2461,7 +2458,7 @@
         <v>53</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
@@ -2472,7 +2469,7 @@
         <v>167</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D12" s="5">
         <v>45642</v>
@@ -2493,7 +2490,7 @@
         <v>170</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
@@ -2504,7 +2501,7 @@
         <v>11</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D13" s="5">
         <v>45628</v>
@@ -2516,16 +2513,16 @@
         <v>45847</v>
       </c>
       <c r="G13" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="H13" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="I13" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>419</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>420</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
@@ -2653,13 +2650,13 @@
         <v>23</v>
       </c>
       <c r="H1" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="I1" s="6" t="s">
-        <v>284</v>
-      </c>
       <c r="J1" s="6" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -2670,7 +2667,7 @@
         <v>182</v>
       </c>
       <c r="C2" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E2" t="s">
         <v>97</v>
@@ -2688,7 +2685,7 @@
         <v>3.1244129975938102</v>
       </c>
       <c r="J2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
@@ -2717,7 +2714,7 @@
         <v>5.6589433976446699</v>
       </c>
       <c r="J3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -2728,7 +2725,7 @@
         <v>133</v>
       </c>
       <c r="C4" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E4" t="s">
         <v>97</v>
@@ -2746,7 +2743,7 @@
         <v>3.1244129975938102</v>
       </c>
       <c r="J4" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -2775,7 +2772,7 @@
         <v>22.9405089971035</v>
       </c>
       <c r="J5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -2786,7 +2783,7 @@
         <v>174</v>
       </c>
       <c r="C6" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E6" t="s">
         <v>43</v>
@@ -2804,7 +2801,7 @@
         <v>13.3017890536159</v>
       </c>
       <c r="J6" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -2833,7 +2830,7 @@
         <v>-0.33822661346496702</v>
       </c>
       <c r="J7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
@@ -2862,7 +2859,7 @@
         <v>17.661905826869599</v>
       </c>
       <c r="J8" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
@@ -2873,7 +2870,7 @@
         <v>177</v>
       </c>
       <c r="C9" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E9" t="s">
         <v>114</v>
@@ -2891,7 +2888,7 @@
         <v>8.0255581112228906</v>
       </c>
       <c r="J9" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
@@ -2920,7 +2917,7 @@
         <v>4.9613980167991301</v>
       </c>
       <c r="J10" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
@@ -2949,7 +2946,7 @@
         <v>22.9405089971035</v>
       </c>
       <c r="J11" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
@@ -2978,7 +2975,7 @@
         <v>8.6098382992801792</v>
       </c>
       <c r="J12" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
@@ -3007,7 +3004,7 @@
         <v>21.415228454744302</v>
       </c>
       <c r="J13" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
@@ -3036,7 +3033,7 @@
         <v>5.6589433976446699</v>
       </c>
       <c r="J14" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
@@ -3065,7 +3062,7 @@
         <v>5.6589433976446699</v>
       </c>
       <c r="J15" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
@@ -3076,7 +3073,7 @@
         <v>182</v>
       </c>
       <c r="C16" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E16" t="s">
         <v>97</v>
@@ -3094,7 +3091,7 @@
         <v>3.1244129975938102</v>
       </c>
       <c r="J16" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
@@ -3123,7 +3120,7 @@
         <v>-0.33822661346496702</v>
       </c>
       <c r="J17" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
@@ -3134,7 +3131,7 @@
         <v>182</v>
       </c>
       <c r="C18" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E18" t="s">
         <v>97</v>
@@ -3152,7 +3149,7 @@
         <v>3.1244129975938102</v>
       </c>
       <c r="J18" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
@@ -3163,7 +3160,7 @@
         <v>133</v>
       </c>
       <c r="C19" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E19" t="s">
         <v>97</v>
@@ -3181,7 +3178,7 @@
         <v>3.1244129975938102</v>
       </c>
       <c r="J19" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
@@ -3210,7 +3207,7 @@
         <v>17.661905826869599</v>
       </c>
       <c r="J20" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
@@ -3239,7 +3236,7 @@
         <v>5.6589433976446699</v>
       </c>
       <c r="J21" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
@@ -3268,7 +3265,7 @@
         <v>4.9613980167991301</v>
       </c>
       <c r="J22" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
@@ -3276,7 +3273,7 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C23" t="s">
         <v>137</v>
@@ -3297,7 +3294,7 @@
         <v>21.415228454744302</v>
       </c>
       <c r="J23" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
@@ -3326,7 +3323,7 @@
         <v>8.6098382992801792</v>
       </c>
       <c r="J24" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
@@ -3355,7 +3352,7 @@
         <v>22.9405089971035</v>
       </c>
       <c r="J25" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
@@ -3384,7 +3381,7 @@
         <v>22.9405089971035</v>
       </c>
       <c r="J26" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
@@ -3413,7 +3410,7 @@
         <v>5.6589433976446699</v>
       </c>
       <c r="J27" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
@@ -3424,7 +3421,7 @@
         <v>177</v>
       </c>
       <c r="C28" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E28" t="s">
         <v>114</v>
@@ -3442,7 +3439,7 @@
         <v>8.0255581112228906</v>
       </c>
       <c r="J28" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
@@ -3453,7 +3450,7 @@
         <v>174</v>
       </c>
       <c r="C29" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E29" t="s">
         <v>43</v>
@@ -3471,7 +3468,7 @@
         <v>13.3017890536159</v>
       </c>
       <c r="J29" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
@@ -3479,19 +3476,19 @@
         <v>3</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C30" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E30" t="s">
+        <v>274</v>
+      </c>
+      <c r="F30" t="s">
         <v>275</v>
       </c>
-      <c r="F30" t="s">
-        <v>276</v>
-      </c>
       <c r="G30" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H30">
         <v>40.633778434327198</v>
@@ -3500,7 +3497,7 @@
         <v>-8.6593167806106006</v>
       </c>
       <c r="J30" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.35">
@@ -3508,19 +3505,19 @@
         <v>3</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="C31" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E31" t="s">
+        <v>274</v>
+      </c>
+      <c r="F31" t="s">
         <v>275</v>
       </c>
-      <c r="F31" t="s">
-        <v>276</v>
-      </c>
       <c r="G31" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H31">
         <v>40.633778434327198</v>
@@ -3529,7 +3526,7 @@
         <v>-8.6593167806106006</v>
       </c>
       <c r="J31" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
@@ -3537,19 +3534,19 @@
         <v>3</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C32" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E32" t="s">
+        <v>274</v>
+      </c>
+      <c r="F32" t="s">
         <v>275</v>
       </c>
-      <c r="F32" t="s">
-        <v>276</v>
-      </c>
       <c r="G32" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H32">
         <v>40.633778434327198</v>
@@ -3558,7 +3555,7 @@
         <v>-8.6593167806106006</v>
       </c>
       <c r="J32" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
@@ -3566,19 +3563,19 @@
         <v>3</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="C33" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E33" t="s">
+        <v>274</v>
+      </c>
+      <c r="F33" t="s">
         <v>275</v>
       </c>
-      <c r="F33" t="s">
-        <v>276</v>
-      </c>
       <c r="G33" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H33">
         <v>40.633778434327198</v>
@@ -3587,7 +3584,7 @@
         <v>-8.6593167806106006</v>
       </c>
       <c r="J33" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.35">
@@ -3595,19 +3592,19 @@
         <v>3</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="C34" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E34" t="s">
+        <v>274</v>
+      </c>
+      <c r="F34" t="s">
         <v>275</v>
       </c>
-      <c r="F34" t="s">
-        <v>276</v>
-      </c>
       <c r="G34" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H34">
         <v>40.633778434327198</v>
@@ -3616,7 +3613,7 @@
         <v>-8.6593167806106006</v>
       </c>
       <c r="J34" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.35">
@@ -3627,16 +3624,16 @@
         <v>187</v>
       </c>
       <c r="C35" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E35" t="s">
+        <v>274</v>
+      </c>
+      <c r="F35" t="s">
         <v>275</v>
       </c>
-      <c r="F35" t="s">
-        <v>276</v>
-      </c>
       <c r="G35" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H35">
         <v>40.633778434327198</v>
@@ -3645,7 +3642,7 @@
         <v>-8.6593167806106006</v>
       </c>
       <c r="J35" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.35">
@@ -3674,7 +3671,7 @@
         <v>-96.347648287433501</v>
       </c>
       <c r="J36" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
@@ -3703,7 +3700,7 @@
         <v>11.342513280116099</v>
       </c>
       <c r="J37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.35">
@@ -3732,7 +3729,7 @@
         <v>-96.347648287433501</v>
       </c>
       <c r="J38" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.35">
@@ -3761,7 +3758,7 @@
         <v>15.468238426254301</v>
       </c>
       <c r="J39" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
@@ -3772,7 +3769,7 @@
         <v>177</v>
       </c>
       <c r="C40" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E40" t="s">
         <v>114</v>
@@ -3790,7 +3787,7 @@
         <v>8.0255581112228906</v>
       </c>
       <c r="J40" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
@@ -3801,16 +3798,16 @@
         <v>186</v>
       </c>
       <c r="C41" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E41" t="s">
+        <v>267</v>
+      </c>
+      <c r="F41" t="s">
         <v>268</v>
       </c>
-      <c r="F41" t="s">
-        <v>269</v>
-      </c>
       <c r="G41" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H41">
         <v>51.6023180801647</v>
@@ -3819,7 +3816,7 @@
         <v>-1.1106435158680901</v>
       </c>
       <c r="J41" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
@@ -3830,13 +3827,13 @@
         <v>172</v>
       </c>
       <c r="C42" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E42" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F42" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G42" t="s">
         <v>89</v>
@@ -3848,7 +3845,7 @@
         <v>4.8657200235795504</v>
       </c>
       <c r="J42" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
@@ -3859,16 +3856,16 @@
         <v>187</v>
       </c>
       <c r="C43" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E43" t="s">
+        <v>274</v>
+      </c>
+      <c r="F43" t="s">
         <v>275</v>
       </c>
-      <c r="F43" t="s">
-        <v>276</v>
-      </c>
       <c r="G43" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H43">
         <v>40.633778434327198</v>
@@ -3877,7 +3874,7 @@
         <v>-8.6593167806106006</v>
       </c>
       <c r="J43" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.35">
@@ -3888,16 +3885,16 @@
         <v>188</v>
       </c>
       <c r="C44" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E44" t="s">
+        <v>267</v>
+      </c>
+      <c r="F44" t="s">
         <v>268</v>
       </c>
-      <c r="F44" t="s">
-        <v>269</v>
-      </c>
       <c r="G44" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H44">
         <v>51.6023180801647</v>
@@ -3906,7 +3903,7 @@
         <v>-1.1106435158680901</v>
       </c>
       <c r="J44" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.35">
@@ -3917,10 +3914,10 @@
         <v>189</v>
       </c>
       <c r="C45" t="s">
+        <v>257</v>
+      </c>
+      <c r="D45" t="s">
         <v>258</v>
-      </c>
-      <c r="D45" t="s">
-        <v>259</v>
       </c>
       <c r="E45" t="s">
         <v>110</v>
@@ -3938,7 +3935,7 @@
         <v>5.66802962647985</v>
       </c>
       <c r="J45" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
@@ -3952,7 +3949,7 @@
         <v>72</v>
       </c>
       <c r="D46" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E46" t="s">
         <v>49</v>
@@ -3970,7 +3967,7 @@
         <v>0.70342542626760896</v>
       </c>
       <c r="J46" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.35">
@@ -3981,10 +3978,10 @@
         <v>191</v>
       </c>
       <c r="C47" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D47" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E47" t="s">
         <v>110</v>
@@ -4002,7 +3999,7 @@
         <v>5.66802962647985</v>
       </c>
       <c r="J47" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
@@ -4013,19 +4010,19 @@
         <v>192</v>
       </c>
       <c r="C48" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D48" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E48" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F48" t="s">
+        <v>270</v>
+      </c>
+      <c r="G48" t="s">
         <v>271</v>
-      </c>
-      <c r="G48" t="s">
-        <v>272</v>
       </c>
       <c r="H48">
         <v>50.736885651002801</v>
@@ -4034,7 +4031,7 @@
         <v>-3.53466898759851</v>
       </c>
       <c r="J48" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
@@ -4045,19 +4042,19 @@
         <v>193</v>
       </c>
       <c r="C49" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D49" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E49" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F49" t="s">
+        <v>270</v>
+      </c>
+      <c r="G49" t="s">
         <v>271</v>
-      </c>
-      <c r="G49" t="s">
-        <v>272</v>
       </c>
       <c r="H49">
         <v>50.736885651002801</v>
@@ -4066,7 +4063,7 @@
         <v>-3.53466898759851</v>
       </c>
       <c r="J49" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.35">
@@ -4077,13 +4074,13 @@
         <v>194</v>
       </c>
       <c r="C50" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D50" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E50" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F50" t="s">
         <v>47</v>
@@ -4098,7 +4095,7 @@
         <v>-0.42133088673402702</v>
       </c>
       <c r="J50" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.35">
@@ -4109,19 +4106,19 @@
         <v>195</v>
       </c>
       <c r="C51" t="s">
+        <v>262</v>
+      </c>
+      <c r="D51" t="s">
         <v>263</v>
       </c>
-      <c r="D51" t="s">
-        <v>264</v>
-      </c>
       <c r="E51" t="s">
+        <v>267</v>
+      </c>
+      <c r="F51" t="s">
         <v>268</v>
       </c>
-      <c r="F51" t="s">
-        <v>269</v>
-      </c>
       <c r="G51" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H51">
         <v>51.6023180801647</v>
@@ -4130,7 +4127,7 @@
         <v>-1.1106435158680901</v>
       </c>
       <c r="J51" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.35">
@@ -4141,10 +4138,10 @@
         <v>196</v>
       </c>
       <c r="C52" t="s">
+        <v>257</v>
+      </c>
+      <c r="D52" t="s">
         <v>258</v>
-      </c>
-      <c r="D52" t="s">
-        <v>259</v>
       </c>
       <c r="E52" t="s">
         <v>110</v>
@@ -4162,7 +4159,7 @@
         <v>5.66802962647985</v>
       </c>
       <c r="J52" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.35">
@@ -4173,13 +4170,13 @@
         <v>197</v>
       </c>
       <c r="C53" t="s">
+        <v>258</v>
+      </c>
+      <c r="D53" t="s">
         <v>259</v>
       </c>
-      <c r="D53" t="s">
-        <v>260</v>
-      </c>
       <c r="E53" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F53" t="s">
         <v>47</v>
@@ -4194,7 +4191,7 @@
         <v>-0.42133088673402702</v>
       </c>
       <c r="J53" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.35">
@@ -4205,10 +4202,10 @@
         <v>198</v>
       </c>
       <c r="C54" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D54" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E54" t="s">
         <v>110</v>
@@ -4226,7 +4223,7 @@
         <v>5.66802962647985</v>
       </c>
       <c r="J54" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
@@ -4237,16 +4234,16 @@
         <v>199</v>
       </c>
       <c r="C55" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E55" t="s">
+        <v>274</v>
+      </c>
+      <c r="F55" t="s">
         <v>275</v>
       </c>
-      <c r="F55" t="s">
-        <v>276</v>
-      </c>
       <c r="G55" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H55">
         <v>40.633778434327198</v>
@@ -4255,7 +4252,7 @@
         <v>-8.6593167806106006</v>
       </c>
       <c r="J55" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.35">
@@ -4266,16 +4263,16 @@
         <v>200</v>
       </c>
       <c r="C56" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E56" t="s">
+        <v>274</v>
+      </c>
+      <c r="F56" t="s">
         <v>275</v>
       </c>
-      <c r="F56" t="s">
-        <v>276</v>
-      </c>
       <c r="G56" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H56">
         <v>40.633778434327198</v>
@@ -4284,7 +4281,7 @@
         <v>-8.6593167806106006</v>
       </c>
       <c r="J56" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.35">
@@ -4295,19 +4292,19 @@
         <v>201</v>
       </c>
       <c r="C57" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D57" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E57" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F57" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="G57" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H57">
         <v>50.1709492732614</v>
@@ -4316,7 +4313,7 @@
         <v>-5.12797037352746</v>
       </c>
       <c r="J57" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.35">
@@ -4327,10 +4324,10 @@
         <v>202</v>
       </c>
       <c r="C58" t="s">
+        <v>265</v>
+      </c>
+      <c r="D58" t="s">
         <v>266</v>
-      </c>
-      <c r="D58" t="s">
-        <v>267</v>
       </c>
       <c r="E58" t="s">
         <v>110</v>
@@ -4348,7 +4345,7 @@
         <v>5.6680081688096902</v>
       </c>
       <c r="J58" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.35">
@@ -4359,19 +4356,19 @@
         <v>203</v>
       </c>
       <c r="C59" t="s">
+        <v>262</v>
+      </c>
+      <c r="D59" t="s">
         <v>263</v>
       </c>
-      <c r="D59" t="s">
-        <v>264</v>
-      </c>
       <c r="E59" t="s">
+        <v>267</v>
+      </c>
+      <c r="F59" t="s">
         <v>268</v>
       </c>
-      <c r="F59" t="s">
-        <v>269</v>
-      </c>
       <c r="G59" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H59">
         <v>51.6023180801647</v>
@@ -4380,7 +4377,7 @@
         <v>-1.1106435158680901</v>
       </c>
       <c r="J59" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.35">
@@ -4391,10 +4388,10 @@
         <v>204</v>
       </c>
       <c r="C60" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D60" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E60" t="s">
         <v>110</v>
@@ -4412,7 +4409,7 @@
         <v>5.66802962647985</v>
       </c>
       <c r="J60" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.35">
@@ -4423,19 +4420,19 @@
         <v>205</v>
       </c>
       <c r="C61" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D61" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E61" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F61" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="G61" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="H61">
         <v>55.683616997457598</v>
@@ -4444,7 +4441,7 @@
         <v>12.5446980519812</v>
       </c>
       <c r="J61" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.35">
@@ -4455,16 +4452,16 @@
         <v>206</v>
       </c>
       <c r="C62" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E62" t="s">
+        <v>267</v>
+      </c>
+      <c r="F62" t="s">
         <v>268</v>
       </c>
-      <c r="F62" t="s">
-        <v>269</v>
-      </c>
       <c r="G62" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H62">
         <v>51.6023180801647</v>
@@ -4473,7 +4470,7 @@
         <v>-1.1106435158680901</v>
       </c>
       <c r="J62" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.35">
@@ -4484,13 +4481,13 @@
         <v>163</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E63" t="s">
         <v>140</v>
       </c>
       <c r="F63" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G63" t="s">
         <v>142</v>
@@ -4502,7 +4499,7 @@
         <v>13.0758769065196</v>
       </c>
       <c r="J63" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
@@ -4513,13 +4510,13 @@
         <v>171</v>
       </c>
       <c r="C64" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E64" t="s">
+        <v>313</v>
+      </c>
+      <c r="F64" t="s">
         <v>314</v>
-      </c>
-      <c r="F64" t="s">
-        <v>315</v>
       </c>
       <c r="G64" t="s">
         <v>30</v>
@@ -4531,7 +4528,7 @@
         <v>-8.6840565629510902</v>
       </c>
       <c r="J64" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.35">
@@ -4542,7 +4539,7 @@
         <v>207</v>
       </c>
       <c r="C65" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E65" t="s">
         <v>37</v>
@@ -4560,7 +4557,7 @@
         <v>11.342090963931099</v>
       </c>
       <c r="J65" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.35">
@@ -4571,7 +4568,7 @@
         <v>208</v>
       </c>
       <c r="C66" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E66" t="s">
         <v>97</v>
@@ -4589,7 +4586,7 @@
         <v>3.1244129975938102</v>
       </c>
       <c r="J66" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.35">
@@ -4600,7 +4597,7 @@
         <v>174</v>
       </c>
       <c r="C67" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E67" t="s">
         <v>43</v>
@@ -4618,7 +4615,7 @@
         <v>13.3017890536159</v>
       </c>
       <c r="J67" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.35">
@@ -4629,7 +4626,7 @@
         <v>209</v>
       </c>
       <c r="C68" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E68" t="s">
         <v>43</v>
@@ -4647,7 +4644,7 @@
         <v>13.3017890536159</v>
       </c>
       <c r="J68" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.35">
@@ -4658,7 +4655,7 @@
         <v>210</v>
       </c>
       <c r="C69" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E69" t="s">
         <v>43</v>
@@ -4676,7 +4673,7 @@
         <v>13.3017890536159</v>
       </c>
       <c r="J69" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.35">
@@ -4687,13 +4684,13 @@
         <v>211</v>
       </c>
       <c r="C70" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E70" t="s">
+        <v>318</v>
+      </c>
+      <c r="F70" t="s">
         <v>319</v>
-      </c>
-      <c r="F70" t="s">
-        <v>320</v>
       </c>
       <c r="G70" t="s">
         <v>26</v>
@@ -4705,7 +4702,7 @@
         <v>7.9613930427179396</v>
       </c>
       <c r="J70" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.35">
@@ -4734,7 +4731,7 @@
         <v>11.342513280116099</v>
       </c>
       <c r="J71" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.35">
@@ -4745,16 +4742,16 @@
         <v>158</v>
       </c>
       <c r="C72" t="s">
+        <v>397</v>
+      </c>
+      <c r="E72" t="s">
         <v>398</v>
       </c>
-      <c r="E72" t="s">
-        <v>399</v>
-      </c>
       <c r="F72" t="s">
+        <v>394</v>
+      </c>
+      <c r="G72" t="s">
         <v>395</v>
-      </c>
-      <c r="G72" t="s">
-        <v>396</v>
       </c>
       <c r="H72">
         <v>46.776582771125803</v>
@@ -4763,7 +4760,7 @@
         <v>-71.276988173455095</v>
       </c>
       <c r="J72" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.35">
@@ -4774,16 +4771,16 @@
         <v>159</v>
       </c>
       <c r="C73" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="D73" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E73" t="s">
+        <v>399</v>
+      </c>
+      <c r="F73" t="s">
         <v>400</v>
-      </c>
-      <c r="F73" t="s">
-        <v>401</v>
       </c>
       <c r="G73" t="s">
         <v>26</v>
@@ -4795,7 +4792,7 @@
         <v>8.6755667843876694</v>
       </c>
       <c r="J73" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.35">
@@ -4824,7 +4821,7 @@
         <v>9.2339481921137203</v>
       </c>
       <c r="J74" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.35">
@@ -4853,7 +4850,7 @@
         <v>11.342513280116099</v>
       </c>
       <c r="J75" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.35">
@@ -4864,7 +4861,7 @@
         <v>162</v>
       </c>
       <c r="C76" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E76" t="s">
         <v>155</v>
@@ -4882,7 +4879,7 @@
         <v>4.9610030976058503</v>
       </c>
       <c r="J76" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.35">
@@ -4911,7 +4908,7 @@
         <v>8.8486790473029</v>
       </c>
       <c r="J77" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.35">
@@ -4940,7 +4937,7 @@
         <v>0.70342542626760896</v>
       </c>
       <c r="J78" s="3" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.35">
@@ -4969,7 +4966,7 @@
         <v>9.2339481921137203</v>
       </c>
       <c r="J79" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.35">
@@ -4998,7 +4995,7 @@
         <v>8.5441549372419008</v>
       </c>
       <c r="J80" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.35">
@@ -5027,7 +5024,7 @@
         <v>8.8486790473029</v>
       </c>
       <c r="J81" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.35">
@@ -5056,7 +5053,7 @@
         <v>9.2339481921137203</v>
       </c>
       <c r="J82" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.35">
@@ -5085,7 +5082,7 @@
         <v>9.2339481921137203</v>
       </c>
       <c r="J83" s="3" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.35">
@@ -5114,7 +5111,7 @@
         <v>8.8486790473029</v>
       </c>
       <c r="J84" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.35">
@@ -5125,7 +5122,7 @@
         <v>220</v>
       </c>
       <c r="C85" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E85" t="s">
         <v>93</v>
@@ -5143,7 +5140,7 @@
         <v>1.5242952647465</v>
       </c>
       <c r="J85" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.35">
@@ -5172,7 +5169,7 @@
         <v>12.3870242893354</v>
       </c>
       <c r="J86" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.35">
@@ -5201,7 +5198,7 @@
         <v>0.70342542626760896</v>
       </c>
       <c r="J87" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.35">
@@ -5233,7 +5230,7 @@
         <v>35.575710739213001</v>
       </c>
       <c r="J88" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.35">
@@ -5262,7 +5259,7 @@
         <v>9.2339481921137203</v>
       </c>
       <c r="J89" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.35">
@@ -5294,7 +5291,7 @@
         <v>9.2339481921137203</v>
       </c>
       <c r="J90" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.35">
@@ -5326,7 +5323,7 @@
         <v>8.8486790473029</v>
       </c>
       <c r="J91" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.35">
@@ -5355,7 +5352,7 @@
         <v>5.6680296141793498</v>
       </c>
       <c r="J92" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.35">
@@ -5384,7 +5381,7 @@
         <v>8.5441515169965392</v>
       </c>
       <c r="J93" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.35">
@@ -5413,7 +5410,7 @@
         <v>5.6680296141793498</v>
       </c>
       <c r="J94" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.35">
@@ -5442,7 +5439,7 @@
         <v>1.5242988815479801</v>
       </c>
       <c r="J95" s="3" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.35">
@@ -5471,7 +5468,7 @@
         <v>21.415228454744302</v>
       </c>
       <c r="J96" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.35">
@@ -5500,7 +5497,7 @@
         <v>5.6589433976446699</v>
       </c>
       <c r="J97" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.35">
@@ -5511,7 +5508,7 @@
         <v>177</v>
       </c>
       <c r="C98" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E98" t="s">
         <v>114</v>
@@ -5529,7 +5526,7 @@
         <v>8.0255581112228906</v>
       </c>
       <c r="J98" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.35">
@@ -5558,7 +5555,7 @@
         <v>7.58964341545685</v>
       </c>
       <c r="J99" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.35">
@@ -5587,7 +5584,7 @@
         <v>22.9405089971035</v>
       </c>
       <c r="J100" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.35">
@@ -5616,7 +5613,7 @@
         <v>-0.33822661346496702</v>
       </c>
       <c r="J101" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.35">
@@ -5645,7 +5642,7 @@
         <v>-0.33822661346496702</v>
       </c>
       <c r="J102" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.35">
@@ -5674,7 +5671,7 @@
         <v>5.6680296141793498</v>
       </c>
       <c r="J103" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.35">
@@ -5703,7 +5700,7 @@
         <v>3.1195775975955802</v>
       </c>
       <c r="J104" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.35">
@@ -5714,7 +5711,7 @@
         <v>174</v>
       </c>
       <c r="C105" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E105" t="s">
         <v>43</v>
@@ -5732,7 +5729,7 @@
         <v>13.3017890536159</v>
       </c>
       <c r="J105" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.35">
@@ -5761,7 +5758,7 @@
         <v>7.58964341545685</v>
       </c>
       <c r="J106" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.35">
@@ -5790,7 +5787,7 @@
         <v>13.0125776148264</v>
       </c>
       <c r="J107" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.35">
@@ -5804,13 +5801,13 @@
         <v>244</v>
       </c>
       <c r="E108" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F108" t="s">
         <v>250</v>
       </c>
       <c r="G108" t="s">
-        <v>252</v>
+        <v>28</v>
       </c>
       <c r="H108">
         <v>42.724137729274403</v>
@@ -5819,7 +5816,7 @@
         <v>-84.479665770414002</v>
       </c>
       <c r="J108" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.35">
@@ -5848,7 +5845,7 @@
         <v>7.58964341545685</v>
       </c>
       <c r="J109" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.35">
@@ -5868,7 +5865,7 @@
         <v>251</v>
       </c>
       <c r="G110" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="H110">
         <v>52.246064944967699</v>
@@ -5877,7 +5874,7 @@
         <v>-7.1386928412645201</v>
       </c>
       <c r="J110" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.35">
@@ -5906,7 +5903,7 @@
         <v>7.58958766603818</v>
       </c>
       <c r="J111" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.35">
@@ -5935,7 +5932,7 @@
         <v>7.58958766603818</v>
       </c>
       <c r="J112" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.35">
@@ -5964,7 +5961,7 @@
         <v>13.0125776148264</v>
       </c>
       <c r="J113" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.35">
@@ -5975,7 +5972,7 @@
         <v>177</v>
       </c>
       <c r="C114" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E114" t="s">
         <v>114</v>
@@ -5993,7 +5990,7 @@
         <v>8.0255581112228906</v>
       </c>
       <c r="J114" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.35">
@@ -6025,7 +6022,7 @@
         <v>13.0125776148264</v>
       </c>
       <c r="J115" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.35">
@@ -6054,7 +6051,7 @@
         <v>7.58958766603818</v>
       </c>
       <c r="J116" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.35">
@@ -6065,7 +6062,7 @@
         <v>177</v>
       </c>
       <c r="C117" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E117" t="s">
         <v>114</v>
@@ -6083,7 +6080,7 @@
         <v>8.0255581112228906</v>
       </c>
       <c r="J117" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.35">
@@ -6091,22 +6088,22 @@
         <v>11</v>
       </c>
       <c r="B118" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C118" t="s">
+        <v>455</v>
+      </c>
+      <c r="D118" t="s">
+        <v>458</v>
+      </c>
+      <c r="E118" t="s">
         <v>456</v>
       </c>
-      <c r="D118" t="s">
-        <v>459</v>
-      </c>
-      <c r="E118" t="s">
+      <c r="F118" t="s">
         <v>457</v>
       </c>
-      <c r="F118" t="s">
-        <v>458</v>
-      </c>
       <c r="G118" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H118">
         <v>52.203154253755997</v>
@@ -6115,7 +6112,7 @@
         <v>0.12090679835312</v>
       </c>
       <c r="J118" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.35">
@@ -6123,16 +6120,16 @@
         <v>11</v>
       </c>
       <c r="B119" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C119" t="s">
+        <v>459</v>
+      </c>
+      <c r="E119" t="s">
         <v>460</v>
       </c>
-      <c r="E119" t="s">
+      <c r="F119" t="s">
         <v>461</v>
-      </c>
-      <c r="F119" t="s">
-        <v>462</v>
       </c>
       <c r="G119" t="s">
         <v>32</v>
@@ -6144,7 +6141,7 @@
         <v>2.4524491101874899</v>
       </c>
       <c r="J119" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.35">
@@ -6152,16 +6149,16 @@
         <v>11</v>
       </c>
       <c r="B120" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C120" t="s">
+        <v>462</v>
+      </c>
+      <c r="E120" t="s">
         <v>463</v>
       </c>
-      <c r="E120" t="s">
+      <c r="F120" t="s">
         <v>464</v>
-      </c>
-      <c r="F120" t="s">
-        <v>465</v>
       </c>
       <c r="G120" t="s">
         <v>26</v>
@@ -6173,7 +6170,7 @@
         <v>10.084835040696399</v>
       </c>
       <c r="J120" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.35">
@@ -6181,16 +6178,16 @@
         <v>11</v>
       </c>
       <c r="B121" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C121" t="s">
+        <v>459</v>
+      </c>
+      <c r="E121" t="s">
         <v>460</v>
       </c>
-      <c r="E121" t="s">
+      <c r="F121" t="s">
         <v>461</v>
-      </c>
-      <c r="F121" t="s">
-        <v>462</v>
       </c>
       <c r="G121" t="s">
         <v>32</v>
@@ -6202,7 +6199,7 @@
         <v>2.4524491101874899</v>
       </c>
       <c r="J121" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="122" spans="1:10" x14ac:dyDescent="0.35">
@@ -6210,19 +6207,19 @@
         <v>11</v>
       </c>
       <c r="B122" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C122" t="s">
+        <v>465</v>
+      </c>
+      <c r="E122" t="s">
         <v>466</v>
       </c>
-      <c r="E122" t="s">
+      <c r="F122" t="s">
         <v>467</v>
       </c>
-      <c r="F122" t="s">
-        <v>468</v>
-      </c>
       <c r="G122" t="s">
-        <v>252</v>
+        <v>28</v>
       </c>
       <c r="H122">
         <v>39.774054222384102</v>
@@ -6231,7 +6228,7 @@
         <v>-86.170761786689695</v>
       </c>
       <c r="J122" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.35">
@@ -6239,19 +6236,19 @@
         <v>11</v>
       </c>
       <c r="B123" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C123" t="s">
+        <v>468</v>
+      </c>
+      <c r="E123" t="s">
         <v>469</v>
       </c>
-      <c r="E123" t="s">
+      <c r="F123" t="s">
         <v>470</v>
       </c>
-      <c r="F123" t="s">
+      <c r="G123" t="s">
         <v>471</v>
-      </c>
-      <c r="G123" t="s">
-        <v>472</v>
       </c>
       <c r="H123">
         <v>60.811112394113501</v>
@@ -6260,7 +6257,7 @@
         <v>23.475501542328999</v>
       </c>
       <c r="J123" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.35">
@@ -6271,7 +6268,7 @@
         <v>174</v>
       </c>
       <c r="C124" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E124" t="s">
         <v>43</v>
@@ -6289,7 +6286,7 @@
         <v>13.3017890536159</v>
       </c>
       <c r="J124" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="125" spans="1:10" x14ac:dyDescent="0.35">
@@ -6297,16 +6294,16 @@
         <v>11</v>
       </c>
       <c r="B125" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C125" t="s">
+        <v>472</v>
+      </c>
+      <c r="E125" t="s">
         <v>473</v>
       </c>
-      <c r="E125" t="s">
+      <c r="F125" t="s">
         <v>474</v>
-      </c>
-      <c r="F125" t="s">
-        <v>475</v>
       </c>
       <c r="G125" t="s">
         <v>89</v>
@@ -6318,7 +6315,7 @@
         <v>6.5380058883133803</v>
       </c>
       <c r="J125" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="126" spans="1:10" x14ac:dyDescent="0.35">
@@ -6329,7 +6326,7 @@
         <v>182</v>
       </c>
       <c r="C126" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E126" t="s">
         <v>97</v>
@@ -6347,7 +6344,7 @@
         <v>3.1244129975938102</v>
       </c>
       <c r="J126" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="127" spans="1:10" x14ac:dyDescent="0.35">
@@ -6355,19 +6352,19 @@
         <v>11</v>
       </c>
       <c r="B127" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C127" t="s">
+        <v>455</v>
+      </c>
+      <c r="E127" t="s">
         <v>456</v>
       </c>
-      <c r="E127" t="s">
+      <c r="F127" t="s">
         <v>457</v>
       </c>
-      <c r="F127" t="s">
-        <v>458</v>
-      </c>
       <c r="G127" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H127">
         <v>52.203154253755997</v>
@@ -6376,7 +6373,7 @@
         <v>0.12090679835312</v>
       </c>
       <c r="J127" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="128" spans="1:10" x14ac:dyDescent="0.35">
@@ -6384,16 +6381,16 @@
         <v>11</v>
       </c>
       <c r="B128" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C128" t="s">
+        <v>459</v>
+      </c>
+      <c r="E128" t="s">
         <v>460</v>
       </c>
-      <c r="E128" t="s">
+      <c r="F128" t="s">
         <v>461</v>
-      </c>
-      <c r="F128" t="s">
-        <v>462</v>
       </c>
       <c r="G128" t="s">
         <v>32</v>
@@ -6405,7 +6402,7 @@
         <v>2.4524491101874899</v>
       </c>
       <c r="J128" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.35">
@@ -6413,16 +6410,16 @@
         <v>11</v>
       </c>
       <c r="B129" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C129" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="E129" t="s">
+        <v>475</v>
+      </c>
+      <c r="F129" t="s">
         <v>476</v>
-      </c>
-      <c r="F129" t="s">
-        <v>477</v>
       </c>
       <c r="G129" t="s">
         <v>30</v>
@@ -6434,7 +6431,7 @@
         <v>2.1960336980134501</v>
       </c>
       <c r="J129" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.35">
@@ -6442,10 +6439,10 @@
         <v>11</v>
       </c>
       <c r="B130" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C130" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="E130" t="s">
         <v>110</v>
@@ -6463,7 +6460,7 @@
         <v>5.6632509764321197</v>
       </c>
       <c r="J130" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.35">
@@ -6471,19 +6468,19 @@
         <v>11</v>
       </c>
       <c r="B131" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C131" t="s">
+        <v>465</v>
+      </c>
+      <c r="E131" t="s">
         <v>466</v>
       </c>
-      <c r="E131" t="s">
+      <c r="F131" t="s">
         <v>467</v>
       </c>
-      <c r="F131" t="s">
-        <v>468</v>
-      </c>
       <c r="G131" t="s">
-        <v>252</v>
+        <v>28</v>
       </c>
       <c r="H131">
         <v>39.774054222384102</v>
@@ -6492,7 +6489,7 @@
         <v>-86.170761786689695</v>
       </c>
       <c r="J131" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.35">
@@ -6500,19 +6497,19 @@
         <v>11</v>
       </c>
       <c r="B132" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="C132" t="s">
+        <v>479</v>
+      </c>
+      <c r="E132" t="s">
         <v>480</v>
       </c>
-      <c r="E132" t="s">
+      <c r="F132" t="s">
         <v>481</v>
       </c>
-      <c r="F132" t="s">
+      <c r="G132" t="s">
         <v>482</v>
-      </c>
-      <c r="G132" t="s">
-        <v>483</v>
       </c>
       <c r="H132">
         <v>-33.930661767621103</v>
@@ -6521,7 +6518,7 @@
         <v>18.8654666401459</v>
       </c>
       <c r="J132" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.35">
@@ -6529,19 +6526,19 @@
         <v>11</v>
       </c>
       <c r="B133" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C133" t="s">
+        <v>483</v>
+      </c>
+      <c r="E133" t="s">
         <v>484</v>
       </c>
-      <c r="E133" t="s">
+      <c r="F133" t="s">
         <v>485</v>
       </c>
-      <c r="F133" t="s">
-        <v>486</v>
-      </c>
       <c r="G133" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="H133">
         <v>56.166737254230803</v>
@@ -6550,7 +6547,7 @@
         <v>10.2030475500672</v>
       </c>
       <c r="J133" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.35">
@@ -6558,10 +6555,10 @@
         <v>11</v>
       </c>
       <c r="B134" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C134" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="E134" t="s">
         <v>110</v>
@@ -6579,7 +6576,7 @@
         <v>5.6632470000000001</v>
       </c>
       <c r="J134" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.35">
@@ -6587,22 +6584,22 @@
         <v>11</v>
       </c>
       <c r="B135" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C135" t="s">
+        <v>483</v>
+      </c>
+      <c r="D135" t="s">
+        <v>487</v>
+      </c>
+      <c r="E135" t="s">
         <v>484</v>
       </c>
-      <c r="D135" t="s">
-        <v>488</v>
-      </c>
-      <c r="E135" t="s">
+      <c r="F135" t="s">
         <v>485</v>
       </c>
-      <c r="F135" t="s">
-        <v>486</v>
-      </c>
       <c r="G135" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="H135">
         <v>56.166737254230803</v>
@@ -6611,7 +6608,7 @@
         <v>10.2030475500672</v>
       </c>
       <c r="J135" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.35">
@@ -6619,19 +6616,19 @@
         <v>11</v>
       </c>
       <c r="B136" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C136" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="E136" t="s">
+        <v>488</v>
+      </c>
+      <c r="F136" t="s">
         <v>489</v>
       </c>
-      <c r="F136" t="s">
+      <c r="G136" t="s">
         <v>490</v>
-      </c>
-      <c r="G136" t="s">
-        <v>491</v>
       </c>
       <c r="H136">
         <v>46.060633671089903</v>
@@ -6640,7 +6637,7 @@
         <v>14.5185184981527</v>
       </c>
       <c r="J136" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.35">
@@ -6669,7 +6666,7 @@
         <v>4.9610030976058503</v>
       </c>
       <c r="J137" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.35">
@@ -6698,7 +6695,7 @@
         <v>4.9610030976058503</v>
       </c>
       <c r="J138" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.35">
@@ -6727,7 +6724,7 @@
         <v>4.9613980167991301</v>
       </c>
       <c r="J139" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.35">
@@ -6756,7 +6753,7 @@
         <v>13.0125776148264</v>
       </c>
       <c r="J140" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.35">
@@ -6785,7 +6782,7 @@
         <v>4.9610030976058503</v>
       </c>
       <c r="J141" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.35">
@@ -6796,7 +6793,7 @@
         <v>67</v>
       </c>
       <c r="C142" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D142" t="s">
         <v>84</v>
@@ -6817,7 +6814,7 @@
         <v>7.9530457688421796</v>
       </c>
       <c r="J142" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.35">
@@ -6828,7 +6825,7 @@
         <v>133</v>
       </c>
       <c r="C143" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E143" t="s">
         <v>97</v>
@@ -6846,7 +6843,7 @@
         <v>3.1244129975938102</v>
       </c>
       <c r="J143" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="144" spans="1:10" x14ac:dyDescent="0.35">
@@ -6857,7 +6854,7 @@
         <v>182</v>
       </c>
       <c r="C144" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E144" t="s">
         <v>97</v>
@@ -6875,7 +6872,7 @@
         <v>3.1244129975938102</v>
       </c>
       <c r="J144" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.35">
@@ -6886,7 +6883,7 @@
         <v>232</v>
       </c>
       <c r="C145" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E145" t="s">
         <v>115</v>
@@ -6904,7 +6901,7 @@
         <v>7.9530457688421796</v>
       </c>
       <c r="J145" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.35">
@@ -6933,7 +6930,7 @@
         <v>-0.34418610289270402</v>
       </c>
       <c r="J146" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="147" spans="1:10" x14ac:dyDescent="0.35">
@@ -6962,7 +6959,7 @@
         <v>11.342513280116099</v>
       </c>
       <c r="J147" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="148" spans="1:10" x14ac:dyDescent="0.35">
@@ -6991,7 +6988,7 @@
         <v>-96.347648287433501</v>
       </c>
       <c r="J148" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="149" spans="1:10" x14ac:dyDescent="0.35">
@@ -7002,7 +6999,7 @@
         <v>177</v>
       </c>
       <c r="C149" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E149" t="s">
         <v>114</v>
@@ -7020,7 +7017,7 @@
         <v>8.0255581112228906</v>
       </c>
       <c r="J149" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="150" spans="1:10" x14ac:dyDescent="0.35">
@@ -7049,7 +7046,7 @@
         <v>13.515464457635399</v>
       </c>
       <c r="J150" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
   </sheetData>
@@ -7076,7 +7073,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>17</v>
@@ -7085,7 +7082,7 @@
         <v>34</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>